<commit_message>
fix: Update chart title
[#OCD-4903]
</commit_message>
<xml_diff>
--- a/chpl/chpl-resources/src/main/resources/CriteriaUpToDateChart.xlsx
+++ b/chpl/chpl-resources/src/main/resources/CriteriaUpToDateChart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ekeyk\projects\chpl-api\chpl\chpl-resources\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87AF3B31-305E-41BD-9CDE-42FE1147AF4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AA1D871-D9DE-42C3-B3BD-60F7B73833E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -697,7 +697,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" sz="1800"/>
-              <a:t>Cures Update Criteria</a:t>
+              <a:t>Up-To-Date Criteria</a:t>
             </a:r>
           </a:p>
           <a:p>

</xml_diff>

<commit_message>
fix: Make fully-up-to-date bars blue in chart
[#OCD-4903]
</commit_message>
<xml_diff>
--- a/chpl/chpl-resources/src/main/resources/CriteriaUpToDateChart.xlsx
+++ b/chpl/chpl-resources/src/main/resources/CriteriaUpToDateChart.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ekeyk\projects\chpl-api\chpl\chpl-resources\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AA1D871-D9DE-42C3-B3BD-60F7B73833E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDAE7F56-4365-454D-88E5-AB8EC03AB3D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,6 +16,19 @@
     <sheet name="Data" sheetId="9" r:id="rId1"/>
     <sheet name="Criteria Up-To-Date Chart" sheetId="13" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">Data!$A$2:$A$17</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Data!$B$1</definedName>
+    <definedName name="_xlchart.v1.10" hidden="1">Data!$F$2:$F$17</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Data!$B$2:$B$17</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">Data!$C$1</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">Data!$C$2:$C$17</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">Data!$D$1</definedName>
+    <definedName name="_xlchart.v1.6" hidden="1">Data!$D$2:$D$17</definedName>
+    <definedName name="_xlchart.v1.7" hidden="1">Data!$E$1</definedName>
+    <definedName name="_xlchart.v1.8" hidden="1">Data!$E$2:$E$17</definedName>
+    <definedName name="_xlchart.v1.9" hidden="1">Data!$F$1</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -766,9 +779,9 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent1"/>
+              <a:schemeClr val="accent3"/>
             </a:solidFill>
-            <a:ln w="25400">
+            <a:ln>
               <a:noFill/>
             </a:ln>
             <a:effectLst/>
@@ -909,7 +922,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent3"/>
+              <a:schemeClr val="accent1"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -1654,6 +1667,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1661,7 +1675,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>

</xml_diff>

<commit_message>
fix: Remove b3 data from chart template
[#OCD-5017]
</commit_message>
<xml_diff>
--- a/chpl/chpl-resources/src/main/resources/CriteriaUpToDateChart.xlsx
+++ b/chpl/chpl-resources/src/main/resources/CriteriaUpToDateChart.xlsx
@@ -1,34 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ekeyk\projects\chpl-api\chpl\chpl-resources\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDAE7F56-4365-454D-88E5-AB8EC03AB3D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63C42A0A-BC82-42E8-A805-3DDCC7697F83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="492" yWindow="564" windowWidth="22548" windowHeight="11676" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="9" r:id="rId1"/>
     <sheet name="Criteria Up-To-Date Chart" sheetId="13" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">Data!$A$2:$A$17</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">Data!$B$1</definedName>
-    <definedName name="_xlchart.v1.10" hidden="1">Data!$F$2:$F$17</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">Data!$B$2:$B$17</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">Data!$C$1</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">Data!$C$2:$C$17</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">Data!$D$1</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">Data!$D$2:$D$17</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">Data!$E$1</definedName>
-    <definedName name="_xlchart.v1.8" hidden="1">Data!$E$2:$E$17</definedName>
-    <definedName name="_xlchart.v1.9" hidden="1">Data!$F$1</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -62,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Criteria</t>
   </si>
@@ -74,9 +61,6 @@
   </si>
   <si>
     <t>b2</t>
-  </si>
-  <si>
-    <t>b3</t>
   </si>
   <si>
     <t>b9</t>
@@ -789,9 +773,9 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$A$2:$A$17</c:f>
+              <c:f>Data!$A$2:$A$16</c:f>
               <c:strCache>
-                <c:ptCount val="16"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>a5</c:v>
                 </c:pt>
@@ -808,36 +792,33 @@
                   <c:v>b2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>b3</c:v>
+                  <c:v>b9</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>b9</c:v>
+                  <c:v>c4</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>c4</c:v>
+                  <c:v>e1</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>e1</c:v>
+                  <c:v>f1</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>f1</c:v>
+                  <c:v>f3</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>f3</c:v>
+                  <c:v>f4</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>f4</c:v>
+                  <c:v>f5</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>f5</c:v>
+                  <c:v>g6</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>g6</c:v>
+                  <c:v>g9</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>g9</c:v>
-                </c:pt>
-                <c:pt idx="15">
                   <c:v>g10</c:v>
                 </c:pt>
               </c:strCache>
@@ -845,10 +826,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$B$2:$B$17</c:f>
+              <c:f>Data!$B$2:$B$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -865,36 +846,33 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>428</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
+                  <c:v>499</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>80</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>637</c:v>
+                </c:pt>
+                <c:pt idx="10">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="8">
-                  <c:v>499</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>80</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>637</c:v>
-                </c:pt>
                 <c:pt idx="11">
-                  <c:v>0</c:v>
+                  <c:v>536</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>536</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>100</c:v>
-                </c:pt>
-                <c:pt idx="15">
                   <c:v>100</c:v>
                 </c:pt>
               </c:numCache>
@@ -932,9 +910,9 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$A$2:$A$17</c:f>
+              <c:f>Data!$A$2:$A$16</c:f>
               <c:strCache>
-                <c:ptCount val="16"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>a5</c:v>
                 </c:pt>
@@ -951,36 +929,33 @@
                   <c:v>b2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>b3</c:v>
+                  <c:v>b9</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>b9</c:v>
+                  <c:v>c4</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>c4</c:v>
+                  <c:v>e1</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>e1</c:v>
+                  <c:v>f1</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>f1</c:v>
+                  <c:v>f3</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>f3</c:v>
+                  <c:v>f4</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>f4</c:v>
+                  <c:v>f5</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>f5</c:v>
+                  <c:v>g6</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>g6</c:v>
+                  <c:v>g9</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>g9</c:v>
-                </c:pt>
-                <c:pt idx="15">
                   <c:v>g10</c:v>
                 </c:pt>
               </c:strCache>
@@ -988,10 +963,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$C$2:$C$17</c:f>
+              <c:f>Data!$C$2:$C$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>100</c:v>
                 </c:pt>
@@ -1008,13 +983,13 @@
                   <c:v>527</c:v>
                 </c:pt>
                 <c:pt idx="5">
+                  <c:v>78</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="7">
                   <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>78</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>500</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -1023,21 +998,18 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0</c:v>
+                  <c:v>400</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>400</c:v>
+                  <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>12</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>50</c:v>
-                </c:pt>
-                <c:pt idx="15">
                   <c:v>50</c:v>
                 </c:pt>
               </c:numCache>
@@ -1091,9 +1063,9 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$A$2:$A$17</c:f>
+              <c:f>Data!$A$2:$A$16</c:f>
               <c:strCache>
-                <c:ptCount val="16"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>a5</c:v>
                 </c:pt>
@@ -1110,36 +1082,33 @@
                   <c:v>b2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>b3</c:v>
+                  <c:v>b9</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>b9</c:v>
+                  <c:v>c4</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>c4</c:v>
+                  <c:v>e1</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>e1</c:v>
+                  <c:v>f1</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>f1</c:v>
+                  <c:v>f3</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>f3</c:v>
+                  <c:v>f4</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>f4</c:v>
+                  <c:v>f5</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>f5</c:v>
+                  <c:v>g6</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>g6</c:v>
+                  <c:v>g9</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>g9</c:v>
-                </c:pt>
-                <c:pt idx="15">
                   <c:v>g10</c:v>
                 </c:pt>
               </c:strCache>
@@ -1147,10 +1116,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$E$2:$E$17</c:f>
+              <c:f>Data!$E$2:$E$16</c:f>
               <c:numCache>
                 <c:formatCode>0.00%</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>1</c:v>
                 </c:pt>
@@ -1167,13 +1136,13 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -1182,21 +1151,18 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1</c:v>
+                  <c:v>2.1897810218978103E-2</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2.1897810218978103E-2</c:v>
+                  <c:v>0.33333333333333331</c:v>
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>0.33333333333333331</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.33333333333333331</c:v>
-                </c:pt>
-                <c:pt idx="15">
                   <c:v>0.33333333333333331</c:v>
                 </c:pt>
               </c:numCache>
@@ -1235,9 +1201,9 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$A$2:$A$17</c:f>
+              <c:f>Data!$A$2:$A$16</c:f>
               <c:strCache>
-                <c:ptCount val="16"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>a5</c:v>
                 </c:pt>
@@ -1254,36 +1220,33 @@
                   <c:v>b2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>b3</c:v>
+                  <c:v>b9</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>b9</c:v>
+                  <c:v>c4</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>c4</c:v>
+                  <c:v>e1</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>e1</c:v>
+                  <c:v>f1</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>f1</c:v>
+                  <c:v>f3</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>f3</c:v>
+                  <c:v>f4</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>f4</c:v>
+                  <c:v>f5</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>f5</c:v>
+                  <c:v>g6</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>g6</c:v>
+                  <c:v>g9</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>g9</c:v>
-                </c:pt>
-                <c:pt idx="15">
                   <c:v>g10</c:v>
                 </c:pt>
               </c:strCache>
@@ -1291,10 +1254,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$F$2:$F$17</c:f>
+              <c:f>Data!$F$2:$F$16</c:f>
               <c:numCache>
                 <c:formatCode>0.00%</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -1311,13 +1274,13 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>1</c:v>
@@ -1326,21 +1289,18 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0</c:v>
+                  <c:v>0.97810218978102192</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.97810218978102192</c:v>
+                  <c:v>0.66666666666666663</c:v>
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>0.66666666666666663</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.66666666666666663</c:v>
-                </c:pt>
-                <c:pt idx="15">
                   <c:v>0.66666666666666663</c:v>
                 </c:pt>
               </c:numCache>
@@ -1379,9 +1339,9 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$A$2:$A$17</c:f>
+              <c:f>Data!$A$2:$A$16</c:f>
               <c:strCache>
-                <c:ptCount val="16"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>a5</c:v>
                 </c:pt>
@@ -1398,36 +1358,33 @@
                   <c:v>b2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>b3</c:v>
+                  <c:v>b9</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>b9</c:v>
+                  <c:v>c4</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>c4</c:v>
+                  <c:v>e1</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>e1</c:v>
+                  <c:v>f1</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>f1</c:v>
+                  <c:v>f3</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>f3</c:v>
+                  <c:v>f4</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>f4</c:v>
+                  <c:v>f5</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>f5</c:v>
+                  <c:v>g6</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>g6</c:v>
+                  <c:v>g9</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>g9</c:v>
-                </c:pt>
-                <c:pt idx="15">
                   <c:v>g10</c:v>
                 </c:pt>
               </c:strCache>
@@ -1435,10 +1392,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$D$2:$D$17</c:f>
+              <c:f>Data!$D$2:$D$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="15"/>
                 <c:pt idx="0">
                   <c:v>100</c:v>
                 </c:pt>
@@ -1455,36 +1412,33 @@
                   <c:v>527</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>428</c:v>
+                  <c:v>78</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>78</c:v>
+                  <c:v>500</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>500</c:v>
+                  <c:v>499</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>499</c:v>
+                  <c:v>80</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>80</c:v>
+                  <c:v>637</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>637</c:v>
+                  <c:v>400</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>400</c:v>
+                  <c:v>548</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>548</c:v>
+                  <c:v>150</c:v>
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>150</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>150</c:v>
-                </c:pt>
-                <c:pt idx="15">
                   <c:v>150</c:v>
                 </c:pt>
               </c:numCache>
@@ -2594,7 +2548,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{306EACB4-2C38-409F-952B-D8F0F42049CF}">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
@@ -2612,21 +2566,21 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" t="s">
         <v>20</v>
-      </c>
-      <c r="F1" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -2649,7 +2603,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -2662,17 +2616,17 @@
         <v>100</v>
       </c>
       <c r="E3" s="2">
-        <f t="shared" ref="E3:E17" si="1">(C3/D3)</f>
+        <f t="shared" ref="E3:E16" si="1">(C3/D3)</f>
         <v>1</v>
       </c>
       <c r="F3" s="2">
-        <f t="shared" ref="F3:F17" si="2">B3/D3</f>
+        <f t="shared" ref="F3:F16" si="2">B3/D3</f>
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -2727,7 +2681,7 @@
         <v>527</v>
       </c>
       <c r="D6">
-        <f t="shared" ref="D6:D17" si="3">B6+C6</f>
+        <f t="shared" ref="D6:D16" si="3">B6+C6</f>
         <v>527</v>
       </c>
       <c r="E6" s="2">
@@ -2744,37 +2698,37 @@
         <v>4</v>
       </c>
       <c r="B7">
-        <v>428</v>
+        <v>0</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <v>78</v>
       </c>
       <c r="D7">
         <f t="shared" si="3"/>
-        <v>428</v>
+        <v>78</v>
       </c>
       <c r="E7" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F7" s="2">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="B8">
         <v>0</v>
       </c>
       <c r="C8">
-        <v>78</v>
+        <v>500</v>
       </c>
       <c r="D8">
         <f t="shared" si="3"/>
-        <v>78</v>
+        <v>500</v>
       </c>
       <c r="E8" s="2">
         <f t="shared" si="1"/>
@@ -2787,40 +2741,40 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="B9">
+        <v>499</v>
+      </c>
+      <c r="C9">
         <v>0</v>
-      </c>
-      <c r="C9">
-        <v>500</v>
       </c>
       <c r="D9">
         <f t="shared" si="3"/>
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="E9" s="2">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9" s="2">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="B10">
-        <v>499</v>
+        <v>80</v>
       </c>
       <c r="C10">
         <v>0</v>
       </c>
       <c r="D10">
         <f t="shared" si="3"/>
-        <v>499</v>
+        <v>80</v>
       </c>
       <c r="E10" s="2">
         <f t="shared" si="1"/>
@@ -2836,14 +2790,14 @@
         <v>17</v>
       </c>
       <c r="B11">
-        <v>80</v>
+        <v>637</v>
       </c>
       <c r="C11">
         <v>0</v>
       </c>
       <c r="D11">
         <f t="shared" si="3"/>
-        <v>80</v>
+        <v>637</v>
       </c>
       <c r="E11" s="2">
         <f t="shared" si="1"/>
@@ -2859,45 +2813,45 @@
         <v>18</v>
       </c>
       <c r="B12">
-        <v>637</v>
+        <v>0</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="D12">
         <f t="shared" si="3"/>
-        <v>637</v>
+        <v>400</v>
       </c>
       <c r="E12" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12" s="2">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="B13">
-        <v>0</v>
+        <v>536</v>
       </c>
       <c r="C13">
-        <v>400</v>
+        <v>12</v>
       </c>
       <c r="D13">
         <f t="shared" si="3"/>
-        <v>400</v>
+        <v>548</v>
       </c>
       <c r="E13" s="2">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>2.1897810218978103E-2</v>
       </c>
       <c r="F13" s="2">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.97810218978102192</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
@@ -2905,22 +2859,22 @@
         <v>7</v>
       </c>
       <c r="B14">
-        <v>536</v>
+        <v>100</v>
       </c>
       <c r="C14">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="D14">
         <f t="shared" si="3"/>
-        <v>548</v>
+        <v>150</v>
       </c>
       <c r="E14" s="2">
         <f t="shared" si="1"/>
-        <v>2.1897810218978103E-2</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="F14" s="2">
         <f t="shared" si="2"/>
-        <v>0.97810218978102192</v>
+        <v>0.66666666666666663</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -2965,29 +2919,6 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="F16" s="2">
-        <f t="shared" si="2"/>
-        <v>0.66666666666666663</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B17">
-        <v>100</v>
-      </c>
-      <c r="C17">
-        <v>50</v>
-      </c>
-      <c r="D17">
-        <f t="shared" si="3"/>
-        <v>150</v>
-      </c>
-      <c r="E17" s="2">
-        <f t="shared" si="1"/>
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F17" s="2">
         <f t="shared" si="2"/>
         <v>0.66666666666666663</v>
       </c>

</xml_diff>

<commit_message>
fix: Make y-axis of chart dynamic
The criteria status report chart looks really small with a hardcoded
y-axis max of 1000 if the report if only run against SLI because they
don't have that many listings. Make the chart y-axis dynamic.

[#OCD-5017]
</commit_message>
<xml_diff>
--- a/chpl/chpl-resources/src/main/resources/CriteriaUpToDateChart.xlsx
+++ b/chpl/chpl-resources/src/main/resources/CriteriaUpToDateChart.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ekeyk\projects\chpl-api\chpl\chpl-resources\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63C42A0A-BC82-42E8-A805-3DDCC7697F83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59FB475E-194A-4D7F-983F-64B0089D36AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="492" yWindow="564" windowWidth="22548" windowHeight="11676" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="564" windowWidth="22548" windowHeight="11676" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="9" r:id="rId1"/>
@@ -1519,7 +1519,6 @@
         <c:axId val="1013162992"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="1000"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>

</xml_diff>

<commit_message>
fix: Swap order of blue/gray stacked bars to be consistent
No idea how this got reversed!

[#OCD-5026]
</commit_message>
<xml_diff>
--- a/chpl/chpl-resources/src/main/resources/CriteriaUpToDateChart.xlsx
+++ b/chpl/chpl-resources/src/main/resources/CriteriaUpToDateChart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ekeyk\projects\chpl-api\chpl\chpl-resources\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59FB475E-194A-4D7F-983F-64B0089D36AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{868151C1-4A50-4793-ADDB-0142D54B91E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="564" windowWidth="22548" windowHeight="11676" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -748,8 +748,145 @@
         <c:grouping val="stacked"/>
         <c:varyColors val="0"/>
         <c:ser>
+          <c:idx val="2"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Data!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Fully Up-To-Date</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Data!$A$2:$A$16</c:f>
+              <c:strCache>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>a5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>a12</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>a15</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>b1</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>b2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>b9</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>c4</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>e1</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>f1</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>f3</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>f4</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>f5</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>g6</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>g9</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>g10</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Data!$C$2:$C$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="15"/>
+                <c:pt idx="0">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>527</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>78</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>400</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>50</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-FC60-4B76-9AA3-F9FD5D283A8E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
           <c:idx val="0"/>
-          <c:order val="0"/>
+          <c:order val="1"/>
           <c:tx>
             <c:strRef>
               <c:f>Data!$B$1</c:f>
@@ -881,143 +1018,6 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-EACC-4953-834A-38AF70169156}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Data!$C$1</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Fully Up-To-Date</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent1"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:cat>
-            <c:strRef>
-              <c:f>Data!$A$2:$A$16</c:f>
-              <c:strCache>
-                <c:ptCount val="15"/>
-                <c:pt idx="0">
-                  <c:v>a5</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>a12</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>a15</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>b1</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>b2</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>b9</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>c4</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>e1</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>f1</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>f3</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>f4</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>f5</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>g6</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>g9</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>g10</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Data!$C$2:$C$16</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="15"/>
-                <c:pt idx="0">
-                  <c:v>100</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>100</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>100</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>527</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>78</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>500</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>400</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>12</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>50</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>50</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>50</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-FC60-4B76-9AA3-F9FD5D283A8E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>

</xml_diff>

<commit_message>
fix!: Correctly display % updated in report if criteria not attested
[#OCD-5056]
</commit_message>
<xml_diff>
--- a/chpl/chpl-resources/src/main/resources/CriteriaUpToDateChart.xlsx
+++ b/chpl/chpl-resources/src/main/resources/CriteriaUpToDateChart.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ekeyk\projects\chpl-api\chpl\chpl-resources\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{868151C1-4A50-4793-ADDB-0142D54B91E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C4DDBE5-4B92-4B7B-BB04-8E9673713DD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="564" windowWidth="22548" windowHeight="11676" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -837,7 +837,7 @@
                   <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>100</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -1403,7 +1403,7 @@
                   <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>100</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>546</c:v>
@@ -2592,11 +2592,11 @@
         <v>100</v>
       </c>
       <c r="E2" s="2">
-        <f>(C2/D2)</f>
+        <f>IF(D2 &gt; 0, (C2/D2), 1)</f>
         <v>1</v>
       </c>
       <c r="F2" s="2">
-        <f>B2/D2</f>
+        <f>IF(D2 &gt; 0, B2/D2, 0)</f>
         <v>0</v>
       </c>
     </row>
@@ -2615,11 +2615,11 @@
         <v>100</v>
       </c>
       <c r="E3" s="2">
-        <f t="shared" ref="E3:E16" si="1">(C3/D3)</f>
+        <f>IF(D3 &gt; 0, (C3/D3), 1)</f>
         <v>1</v>
       </c>
       <c r="F3" s="2">
-        <f t="shared" ref="F3:F16" si="2">B3/D3</f>
+        <f>IF(D3 &gt; 0, B3/D3, 0)</f>
         <v>0</v>
       </c>
     </row>
@@ -2631,18 +2631,17 @@
         <v>0</v>
       </c>
       <c r="C4">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="D4">
-        <f t="shared" si="0"/>
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E4" s="2">
-        <f t="shared" si="1"/>
+        <f>IF(D4 &gt; 0, (C4/D4), 1)</f>
         <v>1</v>
       </c>
       <c r="F4" s="2">
-        <f t="shared" si="2"/>
+        <f>IF(D4 &gt; 0, B4/D4, 0)</f>
         <v>0</v>
       </c>
     </row>
@@ -2661,11 +2660,11 @@
         <v>546</v>
       </c>
       <c r="E5" s="2">
-        <f t="shared" si="1"/>
+        <f>IF(D5 &gt; 0, (C5/D5), 1)</f>
         <v>0</v>
       </c>
       <c r="F5" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="F5:F16" si="1">IF(D5 &gt; 0, B5/D5, 0)</f>
         <v>1</v>
       </c>
     </row>
@@ -2680,15 +2679,15 @@
         <v>527</v>
       </c>
       <c r="D6">
-        <f t="shared" ref="D6:D16" si="3">B6+C6</f>
+        <f t="shared" ref="D6:D16" si="2">B6+C6</f>
         <v>527</v>
       </c>
       <c r="E6" s="2">
+        <f t="shared" ref="E6:E16" si="3">IF(D6 &gt; 0, (C6/D6), 1)</f>
+        <v>1</v>
+      </c>
+      <c r="F6" s="2">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="F6" s="2">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -2703,15 +2702,15 @@
         <v>78</v>
       </c>
       <c r="D7">
+        <f t="shared" si="2"/>
+        <v>78</v>
+      </c>
+      <c r="E7" s="2">
         <f t="shared" si="3"/>
-        <v>78</v>
-      </c>
-      <c r="E7" s="2">
+        <v>1</v>
+      </c>
+      <c r="F7" s="2">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="F7" s="2">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -2726,15 +2725,15 @@
         <v>500</v>
       </c>
       <c r="D8">
+        <f t="shared" si="2"/>
+        <v>500</v>
+      </c>
+      <c r="E8" s="2">
         <f t="shared" si="3"/>
-        <v>500</v>
-      </c>
-      <c r="E8" s="2">
+        <v>1</v>
+      </c>
+      <c r="F8" s="2">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="F8" s="2">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -2749,15 +2748,15 @@
         <v>0</v>
       </c>
       <c r="D9">
+        <f t="shared" si="2"/>
+        <v>499</v>
+      </c>
+      <c r="E9" s="2">
         <f t="shared" si="3"/>
-        <v>499</v>
-      </c>
-      <c r="E9" s="2">
+        <v>0</v>
+      </c>
+      <c r="F9" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F9" s="2">
-        <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
@@ -2772,15 +2771,15 @@
         <v>0</v>
       </c>
       <c r="D10">
+        <f t="shared" si="2"/>
+        <v>80</v>
+      </c>
+      <c r="E10" s="2">
         <f t="shared" si="3"/>
-        <v>80</v>
-      </c>
-      <c r="E10" s="2">
+        <v>0</v>
+      </c>
+      <c r="F10" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F10" s="2">
-        <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
@@ -2795,15 +2794,15 @@
         <v>0</v>
       </c>
       <c r="D11">
+        <f t="shared" si="2"/>
+        <v>637</v>
+      </c>
+      <c r="E11" s="2">
         <f t="shared" si="3"/>
-        <v>637</v>
-      </c>
-      <c r="E11" s="2">
+        <v>0</v>
+      </c>
+      <c r="F11" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F11" s="2">
-        <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
@@ -2818,15 +2817,15 @@
         <v>400</v>
       </c>
       <c r="D12">
+        <f t="shared" si="2"/>
+        <v>400</v>
+      </c>
+      <c r="E12" s="2">
         <f t="shared" si="3"/>
-        <v>400</v>
-      </c>
-      <c r="E12" s="2">
+        <v>1</v>
+      </c>
+      <c r="F12" s="2">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="F12" s="2">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -2841,15 +2840,15 @@
         <v>12</v>
       </c>
       <c r="D13">
+        <f t="shared" si="2"/>
+        <v>548</v>
+      </c>
+      <c r="E13" s="2">
         <f t="shared" si="3"/>
-        <v>548</v>
-      </c>
-      <c r="E13" s="2">
+        <v>2.1897810218978103E-2</v>
+      </c>
+      <c r="F13" s="2">
         <f t="shared" si="1"/>
-        <v>2.1897810218978103E-2</v>
-      </c>
-      <c r="F13" s="2">
-        <f t="shared" si="2"/>
         <v>0.97810218978102192</v>
       </c>
     </row>
@@ -2864,15 +2863,15 @@
         <v>50</v>
       </c>
       <c r="D14">
+        <f t="shared" si="2"/>
+        <v>150</v>
+      </c>
+      <c r="E14" s="2">
         <f t="shared" si="3"/>
-        <v>150</v>
-      </c>
-      <c r="E14" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F14" s="2">
         <f t="shared" si="1"/>
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F14" s="2">
-        <f t="shared" si="2"/>
         <v>0.66666666666666663</v>
       </c>
     </row>
@@ -2887,15 +2886,15 @@
         <v>50</v>
       </c>
       <c r="D15">
+        <f t="shared" si="2"/>
+        <v>150</v>
+      </c>
+      <c r="E15" s="2">
         <f t="shared" si="3"/>
-        <v>150</v>
-      </c>
-      <c r="E15" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F15" s="2">
         <f t="shared" si="1"/>
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F15" s="2">
-        <f t="shared" si="2"/>
         <v>0.66666666666666663</v>
       </c>
     </row>
@@ -2910,15 +2909,15 @@
         <v>50</v>
       </c>
       <c r="D16">
+        <f t="shared" si="2"/>
+        <v>150</v>
+      </c>
+      <c r="E16" s="2">
         <f t="shared" si="3"/>
-        <v>150</v>
-      </c>
-      <c r="E16" s="2">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="F16" s="2">
         <f t="shared" si="1"/>
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="F16" s="2">
-        <f t="shared" si="2"/>
         <v>0.66666666666666663</v>
       </c>
     </row>

</xml_diff>

<commit_message>
I forget what this did
[#OCD-5040]
</commit_message>
<xml_diff>
--- a/chpl/chpl-resources/src/main/resources/CriteriaUpToDateChart.xlsx
+++ b/chpl/chpl-resources/src/main/resources/CriteriaUpToDateChart.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ekeyk\projects\chpl-api\chpl\chpl-resources\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C4DDBE5-4B92-4B7B-BB04-8E9673713DD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C2FA11F-3F07-4456-B439-31632B13B53C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="564" windowWidth="22548" windowHeight="11676" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="36" yWindow="0" windowWidth="22548" windowHeight="11676" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="9" r:id="rId1"/>
-    <sheet name="Criteria Up-To-Date Chart" sheetId="13" r:id="rId2"/>
+    <sheet name="Criteria Up-To-Date Chart" sheetId="13" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -752,7 +751,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Data!$C$1</c:f>
+              <c:f>'Criteria Up-To-Date Chart'!$AC$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -773,7 +772,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$A$2:$A$16</c:f>
+              <c:f>'Criteria Up-To-Date Chart'!$AA$2:$AA$16</c:f>
               <c:strCache>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
@@ -826,7 +825,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$C$2:$C$16</c:f>
+              <c:f>'Criteria Up-To-Date Chart'!$AC$2:$AC$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
@@ -889,7 +888,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Data!$B$1</c:f>
+              <c:f>'Criteria Up-To-Date Chart'!$AB$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -910,7 +909,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$A$2:$A$16</c:f>
+              <c:f>'Criteria Up-To-Date Chart'!$AA$2:$AA$16</c:f>
               <c:strCache>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
@@ -963,7 +962,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$B$2:$B$16</c:f>
+              <c:f>'Criteria Up-To-Date Chart'!$AB$2:$AB$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
@@ -1042,7 +1041,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Data!$E$1</c:f>
+              <c:f>'Criteria Up-To-Date Chart'!$AE$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1063,7 +1062,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$A$2:$A$16</c:f>
+              <c:f>'Criteria Up-To-Date Chart'!$AA$2:$AA$16</c:f>
               <c:strCache>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
@@ -1116,7 +1115,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$E$2:$E$16</c:f>
+              <c:f>'Criteria Up-To-Date Chart'!$AE$2:$AE$16</c:f>
               <c:numCache>
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="15"/>
@@ -1180,7 +1179,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>Data!$F$1</c:f>
+              <c:f>'Criteria Up-To-Date Chart'!$AF$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1201,7 +1200,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$A$2:$A$16</c:f>
+              <c:f>'Criteria Up-To-Date Chart'!$AA$2:$AA$16</c:f>
               <c:strCache>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
@@ -1254,7 +1253,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$F$2:$F$16</c:f>
+              <c:f>'Criteria Up-To-Date Chart'!$AF$2:$AF$16</c:f>
               <c:numCache>
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="15"/>
@@ -1318,7 +1317,7 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>Data!$D$1</c:f>
+              <c:f>'Criteria Up-To-Date Chart'!$AD$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1339,7 +1338,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$A$2:$A$16</c:f>
+              <c:f>'Criteria Up-To-Date Chart'!$AA$2:$AA$16</c:f>
               <c:strCache>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
@@ -1392,7 +1391,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$D$2:$D$16</c:f>
+              <c:f>'Criteria Up-To-Date Chart'!$AD$2:$AD$16</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
@@ -2546,392 +2545,383 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{306EACB4-2C38-409F-952B-D8F0F42049CF}">
-  <dimension ref="A1:F16"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AB74D64-8CFE-41E6-86AC-89D49A6C786C}">
+  <dimension ref="AA1:AF16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="33.33203125" customWidth="1"/>
-    <col min="4" max="4" width="20.88671875" customWidth="1"/>
-    <col min="5" max="5" width="12.21875" customWidth="1"/>
-    <col min="6" max="6" width="13" customWidth="1"/>
+    <col min="27" max="27" width="7" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="20" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="11.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="27:32" x14ac:dyDescent="0.3">
+      <c r="AA1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="AB1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="AC1" t="s">
         <v>11</v>
       </c>
-      <c r="D1" t="s">
+      <c r="AD1" t="s">
         <v>10</v>
       </c>
-      <c r="E1" t="s">
+      <c r="AE1" t="s">
         <v>19</v>
       </c>
-      <c r="F1" t="s">
+      <c r="AF1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="27:32" x14ac:dyDescent="0.3">
+      <c r="AA2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B2">
+      <c r="AB2">
         <v>0</v>
       </c>
-      <c r="C2">
+      <c r="AC2">
         <v>100</v>
       </c>
-      <c r="D2">
-        <f t="shared" ref="D2:D4" si="0">B2+C2</f>
+      <c r="AD2">
+        <f t="shared" ref="AD2:AD3" si="0">AB2+AC2</f>
         <v>100</v>
       </c>
-      <c r="E2" s="2">
-        <f>IF(D2 &gt; 0, (C2/D2), 1)</f>
+      <c r="AE2" s="2">
+        <f>IF(AD2 &gt; 0, (AC2/AD2), 1)</f>
         <v>1</v>
       </c>
-      <c r="F2" s="2">
-        <f>IF(D2 &gt; 0, B2/D2, 0)</f>
+      <c r="AF2" s="2">
+        <f>IF(AD2 &gt; 0, AB2/AD2, 0)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="27:32" x14ac:dyDescent="0.3">
+      <c r="AA3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B3">
+      <c r="AB3">
         <v>0</v>
       </c>
-      <c r="C3">
+      <c r="AC3">
         <v>100</v>
       </c>
-      <c r="D3">
+      <c r="AD3">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="E3" s="2">
-        <f>IF(D3 &gt; 0, (C3/D3), 1)</f>
+      <c r="AE3" s="2">
+        <f>IF(AD3 &gt; 0, (AC3/AD3), 1)</f>
         <v>1</v>
       </c>
-      <c r="F3" s="2">
-        <f>IF(D3 &gt; 0, B3/D3, 0)</f>
+      <c r="AF3" s="2">
+        <f>IF(AD3 &gt; 0, AB3/AD3, 0)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="27:32" x14ac:dyDescent="0.3">
+      <c r="AA4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B4">
+      <c r="AB4">
         <v>0</v>
       </c>
-      <c r="C4">
+      <c r="AC4">
         <v>0</v>
       </c>
-      <c r="D4">
+      <c r="AD4">
         <v>0</v>
       </c>
-      <c r="E4" s="2">
-        <f>IF(D4 &gt; 0, (C4/D4), 1)</f>
+      <c r="AE4" s="2">
+        <f>IF(AD4 &gt; 0, (AC4/AD4), 1)</f>
         <v>1</v>
       </c>
-      <c r="F4" s="2">
-        <f>IF(D4 &gt; 0, B4/D4, 0)</f>
+      <c r="AF4" s="2">
+        <f>IF(AD4 &gt; 0, AB4/AD4, 0)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="27:32" x14ac:dyDescent="0.3">
+      <c r="AA5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B5">
+      <c r="AB5">
         <v>546</v>
       </c>
-      <c r="C5">
+      <c r="AC5">
         <v>0</v>
       </c>
-      <c r="D5">
-        <f>B5+C5</f>
+      <c r="AD5">
+        <f>AB5+AC5</f>
         <v>546</v>
       </c>
-      <c r="E5" s="2">
-        <f>IF(D5 &gt; 0, (C5/D5), 1)</f>
+      <c r="AE5" s="2">
+        <f>IF(AD5 &gt; 0, (AC5/AD5), 1)</f>
         <v>0</v>
       </c>
-      <c r="F5" s="2">
-        <f t="shared" ref="F5:F16" si="1">IF(D5 &gt; 0, B5/D5, 0)</f>
+      <c r="AF5" s="2">
+        <f t="shared" ref="AF5:AF16" si="1">IF(AD5 &gt; 0, AB5/AD5, 0)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="27:32" x14ac:dyDescent="0.3">
+      <c r="AA6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B6">
+      <c r="AB6">
         <v>0</v>
       </c>
-      <c r="C6">
+      <c r="AC6">
         <v>527</v>
       </c>
-      <c r="D6">
-        <f t="shared" ref="D6:D16" si="2">B6+C6</f>
+      <c r="AD6">
+        <f t="shared" ref="AD6:AD16" si="2">AB6+AC6</f>
         <v>527</v>
       </c>
-      <c r="E6" s="2">
-        <f t="shared" ref="E6:E16" si="3">IF(D6 &gt; 0, (C6/D6), 1)</f>
+      <c r="AE6" s="2">
+        <f t="shared" ref="AE6:AE16" si="3">IF(AD6 &gt; 0, (AC6/AD6), 1)</f>
         <v>1</v>
       </c>
-      <c r="F6" s="2">
+      <c r="AF6" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="27:32" x14ac:dyDescent="0.3">
+      <c r="AA7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B7">
+      <c r="AB7">
         <v>0</v>
       </c>
-      <c r="C7">
+      <c r="AC7">
         <v>78</v>
       </c>
-      <c r="D7">
+      <c r="AD7">
         <f t="shared" si="2"/>
         <v>78</v>
       </c>
-      <c r="E7" s="2">
+      <c r="AE7" s="2">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F7" s="2">
+      <c r="AF7" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+    <row r="8" spans="27:32" x14ac:dyDescent="0.3">
+      <c r="AA8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B8">
+      <c r="AB8">
         <v>0</v>
       </c>
-      <c r="C8">
+      <c r="AC8">
         <v>500</v>
       </c>
-      <c r="D8">
+      <c r="AD8">
         <f t="shared" si="2"/>
         <v>500</v>
       </c>
-      <c r="E8" s="2">
+      <c r="AE8" s="2">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F8" s="2">
+      <c r="AF8" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+    <row r="9" spans="27:32" x14ac:dyDescent="0.3">
+      <c r="AA9" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B9">
+      <c r="AB9">
         <v>499</v>
       </c>
-      <c r="C9">
+      <c r="AC9">
         <v>0</v>
       </c>
-      <c r="D9">
+      <c r="AD9">
         <f t="shared" si="2"/>
         <v>499</v>
       </c>
-      <c r="E9" s="2">
+      <c r="AE9" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F9" s="2">
+      <c r="AF9" s="2">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
+    <row r="10" spans="27:32" x14ac:dyDescent="0.3">
+      <c r="AA10" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B10">
+      <c r="AB10">
         <v>80</v>
       </c>
-      <c r="C10">
+      <c r="AC10">
         <v>0</v>
       </c>
-      <c r="D10">
+      <c r="AD10">
         <f t="shared" si="2"/>
         <v>80</v>
       </c>
-      <c r="E10" s="2">
+      <c r="AE10" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F10" s="2">
+      <c r="AF10" s="2">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
+    <row r="11" spans="27:32" x14ac:dyDescent="0.3">
+      <c r="AA11" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B11">
+      <c r="AB11">
         <v>637</v>
       </c>
-      <c r="C11">
+      <c r="AC11">
         <v>0</v>
       </c>
-      <c r="D11">
+      <c r="AD11">
         <f t="shared" si="2"/>
         <v>637</v>
       </c>
-      <c r="E11" s="2">
+      <c r="AE11" s="2">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F11" s="2">
+      <c r="AF11" s="2">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+    <row r="12" spans="27:32" x14ac:dyDescent="0.3">
+      <c r="AA12" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B12">
+      <c r="AB12">
         <v>0</v>
       </c>
-      <c r="C12">
+      <c r="AC12">
         <v>400</v>
       </c>
-      <c r="D12">
+      <c r="AD12">
         <f t="shared" si="2"/>
         <v>400</v>
       </c>
-      <c r="E12" s="2">
+      <c r="AE12" s="2">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F12" s="2">
+      <c r="AF12" s="2">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
+    <row r="13" spans="27:32" x14ac:dyDescent="0.3">
+      <c r="AA13" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B13">
+      <c r="AB13">
         <v>536</v>
       </c>
-      <c r="C13">
+      <c r="AC13">
         <v>12</v>
       </c>
-      <c r="D13">
+      <c r="AD13">
         <f t="shared" si="2"/>
         <v>548</v>
       </c>
-      <c r="E13" s="2">
+      <c r="AE13" s="2">
         <f t="shared" si="3"/>
         <v>2.1897810218978103E-2</v>
       </c>
-      <c r="F13" s="2">
+      <c r="AF13" s="2">
         <f t="shared" si="1"/>
         <v>0.97810218978102192</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
+    <row r="14" spans="27:32" x14ac:dyDescent="0.3">
+      <c r="AA14" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B14">
+      <c r="AB14">
         <v>100</v>
       </c>
-      <c r="C14">
+      <c r="AC14">
         <v>50</v>
       </c>
-      <c r="D14">
+      <c r="AD14">
         <f t="shared" si="2"/>
         <v>150</v>
       </c>
-      <c r="E14" s="2">
+      <c r="AE14" s="2">
         <f t="shared" si="3"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="F14" s="2">
+      <c r="AF14" s="2">
         <f t="shared" si="1"/>
         <v>0.66666666666666663</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
+    <row r="15" spans="27:32" x14ac:dyDescent="0.3">
+      <c r="AA15" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B15">
+      <c r="AB15">
         <v>100</v>
       </c>
-      <c r="C15">
+      <c r="AC15">
         <v>50</v>
       </c>
-      <c r="D15">
+      <c r="AD15">
         <f t="shared" si="2"/>
         <v>150</v>
       </c>
-      <c r="E15" s="2">
+      <c r="AE15" s="2">
         <f t="shared" si="3"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="F15" s="2">
+      <c r="AF15" s="2">
         <f t="shared" si="1"/>
         <v>0.66666666666666663</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
+    <row r="16" spans="27:32" x14ac:dyDescent="0.3">
+      <c r="AA16" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B16">
+      <c r="AB16">
         <v>100</v>
       </c>
-      <c r="C16">
+      <c r="AC16">
         <v>50</v>
       </c>
-      <c r="D16">
+      <c r="AD16">
         <f t="shared" si="2"/>
         <v>150</v>
       </c>
-      <c r="E16" s="2">
+      <c r="AE16" s="2">
         <f t="shared" si="3"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="F16" s="2">
+      <c r="AF16" s="2">
         <f t="shared" si="1"/>
         <v>0.66666666666666663</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AB74D64-8CFE-41E6-86AC-89D49A6C786C}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: Write data for other ACBs correctly in up-to-date chart
[#OCD-5040]
</commit_message>
<xml_diff>
--- a/chpl/chpl-resources/src/main/resources/CriteriaUpToDateChart.xlsx
+++ b/chpl/chpl-resources/src/main/resources/CriteriaUpToDateChart.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ekeyk\projects\chpl-api\chpl\chpl-resources\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C2FA11F-3F07-4456-B439-31632B13B53C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83759BFF-2A0C-4FD4-9E71-39D3ECA64434}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="36" yWindow="0" windowWidth="22548" windowHeight="11676" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="384" yWindow="348" windowWidth="22548" windowHeight="11676" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Criteria Up-To-Date Chart" sheetId="13" r:id="rId1"/>

</xml_diff>

<commit_message>
fix: Correctly copy formula in xlsx template for a15
[#OCD-5040]
</commit_message>
<xml_diff>
--- a/chpl/chpl-resources/src/main/resources/CriteriaUpToDateChart.xlsx
+++ b/chpl/chpl-resources/src/main/resources/CriteriaUpToDateChart.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ekeyk\projects\chpl-api\chpl\chpl-resources\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83759BFF-2A0C-4FD4-9E71-39D3ECA64434}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53972F29-2576-40F7-9ED2-42C2948DAD37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="384" yWindow="348" windowWidth="22548" windowHeight="11676" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="48" yWindow="72" windowWidth="22548" windowHeight="11676" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Criteria Up-To-Date Chart" sheetId="13" r:id="rId1"/>
@@ -2588,7 +2588,7 @@
         <v>100</v>
       </c>
       <c r="AD2">
-        <f t="shared" ref="AD2:AD3" si="0">AB2+AC2</f>
+        <f t="shared" ref="AD2" si="0">AB2+AC2</f>
         <v>100</v>
       </c>
       <c r="AE2" s="2">
@@ -2611,7 +2611,7 @@
         <v>100</v>
       </c>
       <c r="AD3">
-        <f t="shared" si="0"/>
+        <f>AB3+AC3</f>
         <v>100</v>
       </c>
       <c r="AE3" s="2">
@@ -2634,6 +2634,7 @@
         <v>0</v>
       </c>
       <c r="AD4">
+        <f>AB4+AC4</f>
         <v>0</v>
       </c>
       <c r="AE4" s="2">

</xml_diff>